<commit_message>
checkpoint: animation built (just works)
</commit_message>
<xml_diff>
--- a/portfolio_data.xlsx
+++ b/portfolio_data.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -545,19 +545,19 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Contact</v>
+        <v>Narrative</v>
       </c>
       <c r="B9" t="str">
-        <v>phone</v>
+        <v>intro_1</v>
       </c>
       <c r="C9" t="str">
-        <v>+91-6268106030</v>
+        <v>I am a passionate Full-Stack Developer and AI Enthusiast with a strong foundation in modern web technologies and deep learning.</v>
       </c>
       <c r="D9" t="str">
-        <v>tel:+916268106030</v>
+        <v/>
       </c>
       <c r="E9" t="str">
-        <v>phone</v>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -565,38 +565,21 @@
         <v>Narrative</v>
       </c>
       <c r="B10" t="str">
-        <v>intro_1</v>
+        <v>intro_2</v>
       </c>
       <c r="C10" t="str">
-        <v>I am a passionate Full-Stack Developer and AI Enthusiast with a strong foundation in modern web technologies and deep learning.</v>
+        <v>My focus is on creating highly attractive, scalable, and modular applications that bridge the gap between complex AI capabilities and intuitive user experiences.</v>
       </c>
       <c r="D10" t="str">
         <v/>
       </c>
       <c r="E10" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Narrative</v>
-      </c>
-      <c r="B11" t="str">
-        <v>intro_2</v>
-      </c>
-      <c r="C11" t="str">
-        <v>My focus is on creating highly attractive, scalable, and modular applications that bridge the gap between complex AI capabilities and intuitive user experiences.</v>
-      </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
-      <c r="E11" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -734,12 +717,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D1"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
feat: add live project links and update specific GitHub repository URLs
</commit_message>
<xml_diff>
--- a/portfolio_data.xlsx
+++ b/portfolio_data.xlsx
@@ -796,10 +796,10 @@
         <v>briefcase</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>https://fund-connect-ai-ux96.vercel.app/</v>
       </c>
       <c r="I2" t="str">
-        <v>https://github.com/AyushDey1029</v>
+        <v>https://github.com/AyushDey1029/FundConnect_AI</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -826,10 +826,10 @@
         <v>message-circle</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>https://vernacular-fd-advisor-revised-1029.vercel.app/</v>
       </c>
       <c r="I3" t="str">
-        <v>https://github.com/AyushDey1029</v>
+        <v>https://github.com/AyushDey1029/vernacular_fd_advisor_revised_1029</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -859,7 +859,7 @@
         <v/>
       </c>
       <c r="I4" t="str">
-        <v>https://github.com/AyushDey1029</v>
+        <v>https://github.com/AyushDey1029/iot-sensor-data-compression-autoencoder</v>
       </c>
     </row>
   </sheetData>

</xml_diff>